<commit_message>
pcb impresso. falta desenvolver codigo temporizaçao para os motores, trocar codigo display para oled i2c
</commit_message>
<xml_diff>
--- a/LABSI/Orçamento de Corrente.xlsx
+++ b/LABSI/Orçamento de Corrente.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utilizador\Desktop\RAFA\UNI\LABSI-LUMINOSIDADE\LABSI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5A0A904-9C6D-4530-B7E2-2D3E6F382216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F5D0C2-E621-4E5C-8862-7D90A4353C6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{018CE03C-3860-4B8A-9409-A71B2F560A3B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Sistema Autónomo de Controlo de Luz de uma divisão</t>
   </si>
@@ -81,6 +81,12 @@
   </si>
   <si>
     <t>Fita led (0,5m)</t>
+  </si>
+  <si>
+    <t>Sistema Repouso -150mA</t>
+  </si>
+  <si>
+    <t>Sistema com 2 Motores a girar- 600mA</t>
   </si>
 </sst>
 </file>
@@ -471,23 +477,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE4ED3FD-9FE2-4EB4-9E96-F5589858ABA5}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="4" width="17.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -500,14 +506,20 @@
       <c r="D4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="G4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D5">
-        <f t="shared" ref="D5:D16" si="0">PRODUCT(B5,C5)</f>
+        <f t="shared" ref="D5:D14" si="0">PRODUCT(B5,C5)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="G5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -522,7 +534,7 @@
         <v>2.8</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -537,7 +549,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -552,7 +564,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -567,22 +579,22 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
       <c r="B10">
-        <v>700</v>
+        <v>200</v>
       </c>
       <c r="C10">
         <v>2</v>
       </c>
       <c r="D10">
         <f t="shared" si="0"/>
-        <v>1400</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -597,7 +609,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -612,7 +624,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -627,25 +639,25 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>14</v>
       </c>
       <c r="B14">
-        <v>1.2</v>
+        <v>340</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14">
         <f t="shared" si="0"/>
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D15">
-        <f>SUM(D6,D14)</f>
-        <v>4</v>
+        <f>SUM(D6:D14)</f>
+        <v>1294.2649999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>